<commit_message>
Worked on the report and did the least squares regression on the data.
</commit_message>
<xml_diff>
--- a/Lab/ServoMotorDataLightDisk.xlsx
+++ b/Lab/ServoMotorDataLightDisk.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\chris\OneDrive\Desktop\UNI\University-Work\EEE4118F\Lab\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\chris\OneDrive\Desktop\EEE4118F-Lab-2026\Lab\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{95638F9D-8A7C-42CA-BD03-2C827BA2D9B4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{586E090C-62A9-4D5E-AECA-E3441A677847}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="11424" yWindow="0" windowWidth="11712" windowHeight="12336" xr2:uid="{81B9C43C-E6ED-4EA8-9813-E782B5D5103F}"/>
+    <workbookView xWindow="-14505" yWindow="-1425" windowWidth="14610" windowHeight="15585" xr2:uid="{81B9C43C-E6ED-4EA8-9813-E782B5D5103F}"/>
   </bookViews>
   <sheets>
     <sheet name="ServoMotorDataLightDisk.CSV" sheetId="1" r:id="rId1"/>
@@ -9075,7 +9075,7 @@
   <cols>
     <col min="6" max="6" width="17.33203125" customWidth="1"/>
     <col min="7" max="8" width="16.6640625" customWidth="1"/>
-    <col min="9" max="9" width="14.109375" customWidth="1"/>
+    <col min="9" max="9" width="17.5546875" customWidth="1"/>
     <col min="12" max="12" width="17.44140625" customWidth="1"/>
     <col min="13" max="13" width="16.44140625" customWidth="1"/>
     <col min="14" max="14" width="15.33203125" customWidth="1"/>

</xml_diff>